<commit_message>
Bottom Board BOM Economization #135 (in progress)
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/eSpark BOM (20 Boards).xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/eSpark BOM (20 Boards).xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="190">
   <si>
     <t>Component list</t>
   </si>
@@ -587,16 +587,28 @@
   </si>
   <si>
     <t>Remarks</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>C69335</t>
+  </si>
+  <si>
+    <t>LCSC</t>
+  </si>
+  <si>
+    <t>C1591</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -719,6 +731,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -985,10 +1005,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1142,6 +1163,10 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1151,12 +1176,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1198,7 +1226,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1497,24 +1525,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.109375" style="25" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="33.42578125" customWidth="1"/>
-    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.85546875" customWidth="1"/>
-    <col min="14" max="15" width="19.140625" customWidth="1"/>
-    <col min="16" max="18" width="29.42578125" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="33.44140625" customWidth="1"/>
+    <col min="11" max="11" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.88671875" customWidth="1"/>
+    <col min="14" max="15" width="19.109375" customWidth="1"/>
+    <col min="16" max="18" width="29.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1525,16 +1553,16 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
-      <c r="Q1" s="58"/>
-      <c r="R1" s="58"/>
-    </row>
-    <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+    </row>
+    <row r="2" spans="1:18" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="46"/>
@@ -1558,7 +1586,7 @@
       <c r="Q2" s="3"/>
       <c r="R2" s="43"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="47"/>
@@ -1580,9 +1608,9 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="59"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R3" s="61"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="47"/>
@@ -1603,10 +1631,10 @@
       <c r="N4" s="6"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
-      <c r="Q4" s="62"/>
-      <c r="R4" s="60"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="Q4" s="59"/>
+      <c r="R4" s="62"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="47"/>
@@ -1627,10 +1655,10 @@
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
-      <c r="Q5" s="62"/>
-      <c r="R5" s="60"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="Q5" s="59"/>
+      <c r="R5" s="62"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="48"/>
@@ -1647,10 +1675,10 @@
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
-      <c r="Q6" s="62"/>
-      <c r="R6" s="60"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="Q6" s="59"/>
+      <c r="R6" s="62"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="49"/>
@@ -1668,9 +1696,9 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="60"/>
-    </row>
-    <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R7" s="62"/>
+    </row>
+    <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="50"/>
@@ -1688,9 +1716,9 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="60"/>
-    </row>
-    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R8" s="62"/>
+    </row>
+    <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -1744,7 +1772,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
       <c r="B10" s="53">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -1768,22 +1796,38 @@
       <c r="H10" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37"/>
+      <c r="I10" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>187</v>
+      </c>
       <c r="K10" s="38" t="s">
         <v>149</v>
       </c>
       <c r="L10" s="37">
         <v>1</v>
       </c>
-      <c r="M10" s="37"/>
-      <c r="N10" s="37"/>
-      <c r="O10" s="37"/>
-      <c r="P10" s="37"/>
-      <c r="Q10" s="41"/>
+      <c r="M10" s="37">
+        <f>L10*20</f>
+        <v>20</v>
+      </c>
+      <c r="N10" s="37">
+        <v>40</v>
+      </c>
+      <c r="O10" s="63" t="s">
+        <v>188</v>
+      </c>
+      <c r="P10" s="37">
+        <v>1.9199999999999998E-2</v>
+      </c>
+      <c r="Q10" s="41">
+        <f>P10*N10</f>
+        <v>0.7679999999999999</v>
+      </c>
       <c r="R10" s="41"/>
     </row>
-    <row r="11" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="53">
         <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
@@ -1807,22 +1851,38 @@
       <c r="H11" s="39" t="s">
         <v>127</v>
       </c>
-      <c r="I11" s="39"/>
-      <c r="J11" s="39"/>
+      <c r="I11" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J11" s="39" t="s">
+        <v>189</v>
+      </c>
       <c r="K11" s="40" t="s">
         <v>150</v>
       </c>
       <c r="L11" s="39">
         <v>19</v>
       </c>
-      <c r="M11" s="39"/>
-      <c r="N11" s="39"/>
-      <c r="O11" s="39"/>
-      <c r="P11" s="39"/>
-      <c r="Q11" s="42"/>
+      <c r="M11" s="39">
+        <f>L11*20</f>
+        <v>380</v>
+      </c>
+      <c r="N11" s="39">
+        <v>400</v>
+      </c>
+      <c r="O11" s="64" t="s">
+        <v>188</v>
+      </c>
+      <c r="P11" s="39">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q11" s="42">
+        <f t="shared" ref="Q11:Q42" si="1">P11*N11</f>
+        <v>0.55999999999999994</v>
+      </c>
       <c r="R11" s="42"/>
     </row>
-    <row r="12" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -1854,14 +1914,20 @@
       <c r="L12" s="37">
         <v>1</v>
       </c>
-      <c r="M12" s="37"/>
+      <c r="M12" s="37">
+        <f t="shared" ref="M11:M42" si="2">L12*20</f>
+        <v>20</v>
+      </c>
       <c r="N12" s="37"/>
       <c r="O12" s="37"/>
       <c r="P12" s="37"/>
-      <c r="Q12" s="41"/>
+      <c r="Q12" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R12" s="41"/>
     </row>
-    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="53">
         <f t="shared" si="0"/>
@@ -1893,14 +1959,20 @@
       <c r="L13" s="39">
         <v>2</v>
       </c>
-      <c r="M13" s="39"/>
+      <c r="M13" s="39">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
       <c r="N13" s="39"/>
       <c r="O13" s="39"/>
       <c r="P13" s="39"/>
-      <c r="Q13" s="42"/>
+      <c r="Q13" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R13" s="42"/>
     </row>
-    <row r="14" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="53">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -1932,14 +2004,20 @@
       <c r="L14" s="37">
         <v>2</v>
       </c>
-      <c r="M14" s="37"/>
+      <c r="M14" s="37">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
       <c r="N14" s="37"/>
       <c r="O14" s="37"/>
       <c r="P14" s="37"/>
-      <c r="Q14" s="41"/>
+      <c r="Q14" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R14" s="41"/>
     </row>
-    <row r="15" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="53">
         <f t="shared" si="0"/>
@@ -1971,14 +2049,20 @@
       <c r="L15" s="39">
         <v>2</v>
       </c>
-      <c r="M15" s="39"/>
+      <c r="M15" s="39">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
       <c r="N15" s="39"/>
       <c r="O15" s="39"/>
       <c r="P15" s="39"/>
-      <c r="Q15" s="42"/>
+      <c r="Q15" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R15" s="42"/>
     </row>
-    <row r="16" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="53">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -2010,14 +2094,20 @@
       <c r="L16" s="37">
         <v>1</v>
       </c>
-      <c r="M16" s="37"/>
+      <c r="M16" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N16" s="37"/>
       <c r="O16" s="37"/>
       <c r="P16" s="37"/>
-      <c r="Q16" s="41"/>
+      <c r="Q16" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R16" s="41"/>
     </row>
-    <row r="17" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="53">
         <f t="shared" si="0"/>
@@ -2049,14 +2139,20 @@
       <c r="L17" s="39">
         <v>1</v>
       </c>
-      <c r="M17" s="39"/>
+      <c r="M17" s="39">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N17" s="39"/>
       <c r="O17" s="39"/>
       <c r="P17" s="39"/>
-      <c r="Q17" s="42"/>
+      <c r="Q17" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R17" s="42"/>
     </row>
-    <row r="18" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="53">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -2088,14 +2184,20 @@
       <c r="L18" s="37">
         <v>2</v>
       </c>
-      <c r="M18" s="37"/>
+      <c r="M18" s="37">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
       <c r="N18" s="37"/>
       <c r="O18" s="37"/>
       <c r="P18" s="37"/>
-      <c r="Q18" s="41"/>
+      <c r="Q18" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R18" s="41"/>
     </row>
-    <row r="19" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="53">
         <f t="shared" si="0"/>
@@ -2127,14 +2229,20 @@
       <c r="L19" s="39">
         <v>1</v>
       </c>
-      <c r="M19" s="39"/>
+      <c r="M19" s="39">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N19" s="39"/>
       <c r="O19" s="39"/>
       <c r="P19" s="39"/>
-      <c r="Q19" s="42"/>
+      <c r="Q19" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R19" s="42"/>
     </row>
-    <row r="20" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="53">
         <f>ROW(B20) - ROW($B$9)</f>
@@ -2166,14 +2274,20 @@
       <c r="L20" s="37">
         <v>4</v>
       </c>
-      <c r="M20" s="37"/>
+      <c r="M20" s="37">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
       <c r="N20" s="37"/>
       <c r="O20" s="37"/>
       <c r="P20" s="37"/>
-      <c r="Q20" s="41"/>
+      <c r="Q20" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R20" s="41"/>
     </row>
-    <row r="21" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="53">
         <f t="shared" si="0"/>
@@ -2205,14 +2319,20 @@
       <c r="L21" s="39">
         <v>1</v>
       </c>
-      <c r="M21" s="39"/>
+      <c r="M21" s="39">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N21" s="39"/>
       <c r="O21" s="39"/>
       <c r="P21" s="39"/>
-      <c r="Q21" s="42"/>
+      <c r="Q21" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R21" s="42"/>
     </row>
-    <row r="22" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="53">
         <f>ROW(B22) - ROW($B$9)</f>
@@ -2244,14 +2364,20 @@
       <c r="L22" s="37">
         <v>1</v>
       </c>
-      <c r="M22" s="37"/>
+      <c r="M22" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N22" s="37"/>
       <c r="O22" s="37"/>
       <c r="P22" s="37"/>
-      <c r="Q22" s="41"/>
+      <c r="Q22" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R22" s="41"/>
     </row>
-    <row r="23" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="53">
         <f t="shared" si="0"/>
@@ -2283,14 +2409,20 @@
       <c r="L23" s="39">
         <v>1</v>
       </c>
-      <c r="M23" s="39"/>
+      <c r="M23" s="39">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N23" s="39"/>
       <c r="O23" s="39"/>
       <c r="P23" s="39"/>
-      <c r="Q23" s="42"/>
+      <c r="Q23" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R23" s="42"/>
     </row>
-    <row r="24" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="53">
         <f>ROW(B24) - ROW($B$9)</f>
@@ -2322,14 +2454,20 @@
       <c r="L24" s="37">
         <v>1</v>
       </c>
-      <c r="M24" s="37"/>
+      <c r="M24" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N24" s="37"/>
       <c r="O24" s="37"/>
       <c r="P24" s="37"/>
-      <c r="Q24" s="41"/>
+      <c r="Q24" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R24" s="41"/>
     </row>
-    <row r="25" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="53">
         <f t="shared" si="0"/>
@@ -2361,14 +2499,20 @@
       <c r="L25" s="39">
         <v>2</v>
       </c>
-      <c r="M25" s="39"/>
+      <c r="M25" s="39">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
       <c r="N25" s="39"/>
       <c r="O25" s="39"/>
       <c r="P25" s="39"/>
-      <c r="Q25" s="42"/>
+      <c r="Q25" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R25" s="42"/>
     </row>
-    <row r="26" spans="1:18" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="53">
         <f>ROW(B26) - ROW($B$9)</f>
@@ -2400,14 +2544,20 @@
       <c r="L26" s="37">
         <v>40</v>
       </c>
-      <c r="M26" s="37"/>
+      <c r="M26" s="37">
+        <f t="shared" si="2"/>
+        <v>800</v>
+      </c>
       <c r="N26" s="37"/>
       <c r="O26" s="37"/>
       <c r="P26" s="37"/>
-      <c r="Q26" s="41"/>
+      <c r="Q26" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R26" s="41"/>
     </row>
-    <row r="27" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="53">
         <f t="shared" si="0"/>
@@ -2439,14 +2589,20 @@
       <c r="L27" s="39">
         <v>7</v>
       </c>
-      <c r="M27" s="39"/>
+      <c r="M27" s="39">
+        <f t="shared" si="2"/>
+        <v>140</v>
+      </c>
       <c r="N27" s="39"/>
       <c r="O27" s="39"/>
       <c r="P27" s="39"/>
-      <c r="Q27" s="42"/>
+      <c r="Q27" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R27" s="42"/>
     </row>
-    <row r="28" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="53">
         <f>ROW(B28) - ROW($B$9)</f>
@@ -2478,14 +2634,20 @@
       <c r="L28" s="37">
         <v>1</v>
       </c>
-      <c r="M28" s="37"/>
+      <c r="M28" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N28" s="37"/>
       <c r="O28" s="37"/>
       <c r="P28" s="37"/>
-      <c r="Q28" s="41"/>
+      <c r="Q28" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R28" s="41"/>
     </row>
-    <row r="29" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="53">
         <f t="shared" si="0"/>
@@ -2517,14 +2679,20 @@
       <c r="L29" s="39">
         <v>2</v>
       </c>
-      <c r="M29" s="39"/>
+      <c r="M29" s="39">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
       <c r="N29" s="39"/>
       <c r="O29" s="39"/>
       <c r="P29" s="39"/>
-      <c r="Q29" s="42"/>
+      <c r="Q29" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R29" s="42"/>
     </row>
-    <row r="30" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
       <c r="B30" s="53">
         <f>ROW(B30) - ROW($B$9)</f>
@@ -2556,14 +2724,20 @@
       <c r="L30" s="37">
         <v>1</v>
       </c>
-      <c r="M30" s="37"/>
+      <c r="M30" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N30" s="37"/>
       <c r="O30" s="37"/>
       <c r="P30" s="37"/>
-      <c r="Q30" s="41"/>
+      <c r="Q30" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R30" s="41"/>
     </row>
-    <row r="31" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
       <c r="B31" s="53">
         <f t="shared" si="0"/>
@@ -2595,14 +2769,20 @@
       <c r="L31" s="39">
         <v>2</v>
       </c>
-      <c r="M31" s="39"/>
+      <c r="M31" s="39">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
       <c r="N31" s="39"/>
       <c r="O31" s="39"/>
       <c r="P31" s="39"/>
-      <c r="Q31" s="42"/>
+      <c r="Q31" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R31" s="42"/>
     </row>
-    <row r="32" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="53">
         <f>ROW(B32) - ROW($B$9)</f>
@@ -2630,14 +2810,20 @@
       <c r="L32" s="37">
         <v>8</v>
       </c>
-      <c r="M32" s="37"/>
+      <c r="M32" s="37">
+        <f t="shared" si="2"/>
+        <v>160</v>
+      </c>
       <c r="N32" s="37"/>
       <c r="O32" s="37"/>
       <c r="P32" s="37"/>
-      <c r="Q32" s="41"/>
+      <c r="Q32" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R32" s="41"/>
     </row>
-    <row r="33" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="53">
         <f t="shared" si="0"/>
@@ -2669,14 +2855,20 @@
       <c r="L33" s="39">
         <v>1</v>
       </c>
-      <c r="M33" s="39"/>
+      <c r="M33" s="39">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N33" s="39"/>
       <c r="O33" s="39"/>
       <c r="P33" s="39"/>
-      <c r="Q33" s="42"/>
+      <c r="Q33" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R33" s="42"/>
     </row>
-    <row r="34" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="53">
         <f>ROW(B34) - ROW($B$9)</f>
@@ -2708,14 +2900,20 @@
       <c r="L34" s="37">
         <v>1</v>
       </c>
-      <c r="M34" s="37"/>
+      <c r="M34" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N34" s="37"/>
       <c r="O34" s="37"/>
       <c r="P34" s="37"/>
-      <c r="Q34" s="41"/>
+      <c r="Q34" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R34" s="41"/>
     </row>
-    <row r="35" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="B35" s="53">
         <f t="shared" si="0"/>
@@ -2747,14 +2945,20 @@
       <c r="L35" s="39">
         <v>1</v>
       </c>
-      <c r="M35" s="39"/>
+      <c r="M35" s="39">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N35" s="39"/>
       <c r="O35" s="39"/>
       <c r="P35" s="39"/>
-      <c r="Q35" s="42"/>
+      <c r="Q35" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R35" s="42"/>
     </row>
-    <row r="36" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1"/>
       <c r="B36" s="53">
         <f>ROW(B36) - ROW($B$9)</f>
@@ -2786,14 +2990,20 @@
       <c r="L36" s="37">
         <v>1</v>
       </c>
-      <c r="M36" s="37"/>
+      <c r="M36" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N36" s="37"/>
       <c r="O36" s="37"/>
       <c r="P36" s="37"/>
-      <c r="Q36" s="41"/>
+      <c r="Q36" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R36" s="41"/>
     </row>
-    <row r="37" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1"/>
       <c r="B37" s="53">
         <f t="shared" si="0"/>
@@ -2825,14 +3035,20 @@
       <c r="L37" s="39">
         <v>1</v>
       </c>
-      <c r="M37" s="39"/>
+      <c r="M37" s="39">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N37" s="39"/>
       <c r="O37" s="39"/>
       <c r="P37" s="39"/>
-      <c r="Q37" s="42"/>
+      <c r="Q37" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R37" s="42"/>
     </row>
-    <row r="38" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
       <c r="B38" s="53">
         <f>ROW(B38) - ROW($B$9)</f>
@@ -2864,14 +3080,20 @@
       <c r="L38" s="37">
         <v>1</v>
       </c>
-      <c r="M38" s="37"/>
+      <c r="M38" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N38" s="37"/>
       <c r="O38" s="37"/>
       <c r="P38" s="37"/>
-      <c r="Q38" s="41"/>
+      <c r="Q38" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R38" s="41"/>
     </row>
-    <row r="39" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1"/>
       <c r="B39" s="53">
         <f t="shared" si="0"/>
@@ -2903,14 +3125,20 @@
       <c r="L39" s="39">
         <v>1</v>
       </c>
-      <c r="M39" s="39"/>
+      <c r="M39" s="39">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N39" s="39"/>
       <c r="O39" s="39"/>
       <c r="P39" s="39"/>
-      <c r="Q39" s="42"/>
+      <c r="Q39" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R39" s="42"/>
     </row>
-    <row r="40" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
       <c r="B40" s="53">
         <f>ROW(B40) - ROW($B$9)</f>
@@ -2942,14 +3170,20 @@
       <c r="L40" s="37">
         <v>1</v>
       </c>
-      <c r="M40" s="37"/>
+      <c r="M40" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N40" s="37"/>
       <c r="O40" s="37"/>
       <c r="P40" s="37"/>
-      <c r="Q40" s="41"/>
+      <c r="Q40" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R40" s="41"/>
     </row>
-    <row r="41" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1"/>
       <c r="B41" s="53">
         <f t="shared" si="0"/>
@@ -2981,14 +3215,20 @@
       <c r="L41" s="39">
         <v>1</v>
       </c>
-      <c r="M41" s="39"/>
+      <c r="M41" s="39">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N41" s="39"/>
       <c r="O41" s="39"/>
       <c r="P41" s="39"/>
-      <c r="Q41" s="42"/>
+      <c r="Q41" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R41" s="42"/>
     </row>
-    <row r="42" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1"/>
       <c r="B42" s="53">
         <f>ROW(B42) - ROW($B$9)</f>
@@ -3013,21 +3253,27 @@
         <v>147</v>
       </c>
       <c r="I42" s="37"/>
-      <c r="J42" s="61"/>
+      <c r="J42" s="58"/>
       <c r="K42" s="38" t="s">
         <v>101</v>
       </c>
       <c r="L42" s="37">
         <v>1</v>
       </c>
-      <c r="M42" s="37"/>
+      <c r="M42" s="37">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="N42" s="37"/>
       <c r="O42" s="37"/>
       <c r="P42" s="37"/>
-      <c r="Q42" s="41"/>
+      <c r="Q42" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R42" s="41"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="32"/>
       <c r="C43" s="51"/>
@@ -3049,7 +3295,7 @@
       <c r="Q43" s="36"/>
       <c r="R43" s="44"/>
     </row>
-    <row r="44" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1"/>
       <c r="B44" s="24"/>
       <c r="C44" s="52"/>
@@ -3076,8 +3322,12 @@
     <mergeCell ref="K1:R1"/>
     <mergeCell ref="R3:R8"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bottom board BOM Economization #135 (Complete)
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/eSpark BOM (20 Boards).xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/eSpark BOM (20 Boards).xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="235">
   <si>
     <t>Component list</t>
   </si>
@@ -599,6 +599,141 @@
   </si>
   <si>
     <t>C1591</t>
+  </si>
+  <si>
+    <t>TAJA105K016RNJ</t>
+  </si>
+  <si>
+    <t>C7174</t>
+  </si>
+  <si>
+    <t>Low cost alternate. Design change needed due to different package size of capacitor</t>
+  </si>
+  <si>
+    <t>C86017</t>
+  </si>
+  <si>
+    <t>C113797</t>
+  </si>
+  <si>
+    <t>UMK063CG100DTHF</t>
+  </si>
+  <si>
+    <t>C2168858</t>
+  </si>
+  <si>
+    <t>C96446</t>
+  </si>
+  <si>
+    <t>PESD2CAN,215</t>
+  </si>
+  <si>
+    <t>C75176</t>
+  </si>
+  <si>
+    <t>Quantity changed from 2/board to 1/board due to 2xdiodes in single package. Design change required</t>
+  </si>
+  <si>
+    <t>C82326</t>
+  </si>
+  <si>
+    <t>Ferrite0603</t>
+  </si>
+  <si>
+    <t>C307770</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>C515365</t>
+  </si>
+  <si>
+    <t>MHT136CGCT</t>
+  </si>
+  <si>
+    <t>C401111</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>C94515</t>
+  </si>
+  <si>
+    <t>C106228</t>
+  </si>
+  <si>
+    <t>C98220</t>
+  </si>
+  <si>
+    <t>0201WMF8060TEE</t>
+  </si>
+  <si>
+    <t>C474262</t>
+  </si>
+  <si>
+    <t>C14676</t>
+  </si>
+  <si>
+    <t>C114669</t>
+  </si>
+  <si>
+    <t>CR0603-FX-57R6ELF</t>
+  </si>
+  <si>
+    <t>C203694</t>
+  </si>
+  <si>
+    <t>DO NOT MOUNT</t>
+  </si>
+  <si>
+    <t>GT-TC025D-H0065-L1</t>
+  </si>
+  <si>
+    <t>C778132</t>
+  </si>
+  <si>
+    <t>STM32F407VET6</t>
+  </si>
+  <si>
+    <t>C28730</t>
+  </si>
+  <si>
+    <t>Design change required. Only symbol change. No PCB or Footprint will change</t>
+  </si>
+  <si>
+    <t>SN65HVDA1040AQDRQ1</t>
+  </si>
+  <si>
+    <t>C188675</t>
+  </si>
+  <si>
+    <t>TLE5012BE1000</t>
+  </si>
+  <si>
+    <t>C123083</t>
+  </si>
+  <si>
+    <t>Design change required. Need approval from client first as this change will lead to firmware changes as well</t>
+  </si>
+  <si>
+    <t>UTSource</t>
+  </si>
+  <si>
+    <t>C100024</t>
+  </si>
+  <si>
+    <t>C233772</t>
+  </si>
+  <si>
+    <t>32.768KHz</t>
+  </si>
+  <si>
+    <t>Total Cost</t>
+  </si>
+  <si>
+    <t>Cost per Board</t>
   </si>
 </sst>
 </file>
@@ -608,7 +743,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -739,8 +874,46 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -771,6 +944,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="21">
     <border>
@@ -1009,7 +1200,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1167,6 +1358,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1176,11 +1373,73 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1553,14 +1812,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
     </row>
     <row r="2" spans="1:18" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -1608,7 +1867,7 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="61"/>
+      <c r="R3" s="63"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -1632,7 +1891,7 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="59"/>
-      <c r="R4" s="62"/>
+      <c r="R4" s="64"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
@@ -1656,7 +1915,7 @@
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
       <c r="Q5" s="59"/>
-      <c r="R5" s="62"/>
+      <c r="R5" s="64"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -1676,7 +1935,7 @@
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
       <c r="Q6" s="59"/>
-      <c r="R6" s="62"/>
+      <c r="R6" s="64"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -1696,7 +1955,7 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="62"/>
+      <c r="R7" s="64"/>
     </row>
     <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
@@ -1716,7 +1975,7 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="62"/>
+      <c r="R8" s="64"/>
     </row>
     <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
@@ -1815,7 +2074,7 @@
       <c r="N10" s="37">
         <v>40</v>
       </c>
-      <c r="O10" s="63" t="s">
+      <c r="O10" s="60" t="s">
         <v>188</v>
       </c>
       <c r="P10" s="37">
@@ -1870,7 +2129,7 @@
       <c r="N11" s="39">
         <v>400</v>
       </c>
-      <c r="O11" s="64" t="s">
+      <c r="O11" s="61" t="s">
         <v>188</v>
       </c>
       <c r="P11" s="39">
@@ -1882,50 +2141,62 @@
       </c>
       <c r="R11" s="42"/>
     </row>
-    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="C12" s="69" t="s">
         <v>164</v>
       </c>
-      <c r="D12" s="37" t="s">
+      <c r="D12" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="38" t="s">
+      <c r="E12" s="70" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="37" t="s">
+      <c r="F12" s="69" t="s">
         <v>175</v>
       </c>
-      <c r="G12" s="38" t="s">
+      <c r="G12" s="70" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="37" t="s">
+      <c r="H12" s="69" t="s">
         <v>128</v>
       </c>
-      <c r="I12" s="37"/>
-      <c r="J12" s="37"/>
-      <c r="K12" s="38" t="s">
+      <c r="I12" s="69" t="s">
+        <v>190</v>
+      </c>
+      <c r="J12" s="69" t="s">
+        <v>191</v>
+      </c>
+      <c r="K12" s="70" t="s">
         <v>151</v>
       </c>
-      <c r="L12" s="37">
+      <c r="L12" s="69">
         <v>1</v>
       </c>
-      <c r="M12" s="37">
-        <f t="shared" ref="M11:M42" si="2">L12*20</f>
+      <c r="M12" s="69">
+        <f t="shared" ref="M12:M42" si="2">L12*20</f>
         <v>20</v>
       </c>
-      <c r="N12" s="37"/>
-      <c r="O12" s="37"/>
-      <c r="P12" s="37"/>
-      <c r="Q12" s="41">
+      <c r="N12" s="69">
+        <v>25</v>
+      </c>
+      <c r="O12" s="71" t="s">
+        <v>188</v>
+      </c>
+      <c r="P12" s="69">
+        <v>6.1499999999999999E-2</v>
+      </c>
+      <c r="Q12" s="72">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R12" s="41"/>
+        <v>1.5375000000000001</v>
+      </c>
+      <c r="R12" s="75" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
@@ -1951,8 +2222,12 @@
       <c r="H13" s="39" t="s">
         <v>129</v>
       </c>
-      <c r="I13" s="39"/>
-      <c r="J13" s="39"/>
+      <c r="I13" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J13" s="39" t="s">
+        <v>193</v>
+      </c>
       <c r="K13" s="40" t="s">
         <v>152</v>
       </c>
@@ -1963,12 +2238,18 @@
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="N13" s="39"/>
-      <c r="O13" s="39"/>
-      <c r="P13" s="39"/>
+      <c r="N13" s="39">
+        <v>50</v>
+      </c>
+      <c r="O13" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P13" s="39">
+        <v>5.0099999999999999E-2</v>
+      </c>
       <c r="Q13" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.5049999999999999</v>
       </c>
       <c r="R13" s="42"/>
     </row>
@@ -1996,8 +2277,12 @@
       <c r="H14" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="I14" s="37"/>
-      <c r="J14" s="37"/>
+      <c r="I14" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>194</v>
+      </c>
       <c r="K14" s="38" t="s">
         <v>153</v>
       </c>
@@ -2008,12 +2293,18 @@
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="N14" s="37"/>
-      <c r="O14" s="37"/>
-      <c r="P14" s="37"/>
+      <c r="N14" s="37">
+        <v>100</v>
+      </c>
+      <c r="O14" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P14" s="37">
+        <v>3.3999999999999998E-3</v>
+      </c>
       <c r="Q14" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.33999999999999997</v>
       </c>
       <c r="R14" s="41"/>
     </row>
@@ -2041,8 +2332,12 @@
       <c r="H15" s="39" t="s">
         <v>131</v>
       </c>
-      <c r="I15" s="39"/>
-      <c r="J15" s="39"/>
+      <c r="I15" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="J15" s="39" t="s">
+        <v>196</v>
+      </c>
       <c r="K15" s="40" t="s">
         <v>154</v>
       </c>
@@ -2053,12 +2348,18 @@
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="N15" s="39"/>
-      <c r="O15" s="39"/>
-      <c r="P15" s="39"/>
+      <c r="N15" s="39">
+        <v>50</v>
+      </c>
+      <c r="O15" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P15" s="39">
+        <v>7.3000000000000001E-3</v>
+      </c>
       <c r="Q15" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.36499999999999999</v>
       </c>
       <c r="R15" s="42"/>
     </row>
@@ -2086,8 +2387,12 @@
       <c r="H16" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="I16" s="37"/>
-      <c r="J16" s="37"/>
+      <c r="I16" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J16" s="37" t="s">
+        <v>197</v>
+      </c>
       <c r="K16" s="38" t="s">
         <v>155</v>
       </c>
@@ -2098,12 +2403,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N16" s="37"/>
-      <c r="O16" s="37"/>
-      <c r="P16" s="37"/>
+      <c r="N16" s="37">
+        <v>40</v>
+      </c>
+      <c r="O16" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P16" s="37">
+        <v>1.49E-2</v>
+      </c>
       <c r="Q16" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.59599999999999997</v>
       </c>
       <c r="R16" s="41"/>
     </row>
@@ -2131,8 +2442,12 @@
       <c r="H17" s="39" t="s">
         <v>127</v>
       </c>
-      <c r="I17" s="39"/>
-      <c r="J17" s="39"/>
+      <c r="I17" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J17" s="39" t="s">
+        <v>189</v>
+      </c>
       <c r="K17" s="40" t="s">
         <v>150</v>
       </c>
@@ -2143,59 +2458,77 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N17" s="39"/>
-      <c r="O17" s="39"/>
-      <c r="P17" s="39"/>
+      <c r="N17" s="39">
+        <v>100</v>
+      </c>
+      <c r="O17" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P17" s="39">
+        <v>1.4E-3</v>
+      </c>
       <c r="Q17" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.13999999999999999</v>
       </c>
       <c r="R17" s="42"/>
     </row>
-    <row r="18" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="53">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="37" t="s">
+      <c r="C18" s="69" t="s">
         <v>165</v>
       </c>
-      <c r="D18" s="37" t="s">
+      <c r="D18" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="38" t="s">
+      <c r="E18" s="70" t="s">
         <v>52</v>
       </c>
-      <c r="F18" s="37" t="s">
+      <c r="F18" s="69" t="s">
         <v>175</v>
       </c>
-      <c r="G18" s="37" t="s">
+      <c r="G18" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="37" t="s">
+      <c r="H18" s="69" t="s">
         <v>132</v>
       </c>
-      <c r="I18" s="37"/>
-      <c r="J18" s="37"/>
-      <c r="K18" s="38" t="s">
-        <v>82</v>
-      </c>
-      <c r="L18" s="37">
-        <v>2</v>
-      </c>
-      <c r="M18" s="37">
+      <c r="I18" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="J18" s="69" t="s">
+        <v>199</v>
+      </c>
+      <c r="K18" s="70" t="s">
+        <v>186</v>
+      </c>
+      <c r="L18" s="74">
+        <v>1</v>
+      </c>
+      <c r="M18" s="69">
         <f t="shared" si="2"/>
-        <v>40</v>
-      </c>
-      <c r="N18" s="37"/>
-      <c r="O18" s="37"/>
-      <c r="P18" s="37"/>
-      <c r="Q18" s="41">
+        <v>20</v>
+      </c>
+      <c r="N18" s="69">
+        <v>25</v>
+      </c>
+      <c r="O18" s="71" t="s">
+        <v>188</v>
+      </c>
+      <c r="P18" s="69">
+        <v>0.17119999999999999</v>
+      </c>
+      <c r="Q18" s="72">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R18" s="41"/>
+        <v>4.2799999999999994</v>
+      </c>
+      <c r="R18" s="75" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="19" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
@@ -2221,10 +2554,14 @@
       <c r="H19" s="39" t="s">
         <v>133</v>
       </c>
-      <c r="I19" s="39"/>
-      <c r="J19" s="39"/>
+      <c r="I19" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J19" s="39" t="s">
+        <v>201</v>
+      </c>
       <c r="K19" s="40" t="s">
-        <v>109</v>
+        <v>186</v>
       </c>
       <c r="L19" s="39">
         <v>1</v>
@@ -2233,12 +2570,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N19" s="39"/>
-      <c r="O19" s="39"/>
-      <c r="P19" s="39"/>
+      <c r="N19" s="39">
+        <v>25</v>
+      </c>
+      <c r="O19" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P19" s="39">
+        <v>0.1066</v>
+      </c>
       <c r="Q19" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.665</v>
       </c>
       <c r="R19" s="42"/>
     </row>
@@ -2258,7 +2601,7 @@
         <v>54</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>84</v>
+        <v>202</v>
       </c>
       <c r="G20" s="38" t="s">
         <v>84</v>
@@ -2266,10 +2609,14 @@
       <c r="H20" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="I20" s="37"/>
-      <c r="J20" s="37"/>
+      <c r="I20" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J20" s="37" t="s">
+        <v>203</v>
+      </c>
       <c r="K20" s="38" t="s">
-        <v>84</v>
+        <v>186</v>
       </c>
       <c r="L20" s="37">
         <v>4</v>
@@ -2278,12 +2625,18 @@
         <f t="shared" si="2"/>
         <v>80</v>
       </c>
-      <c r="N20" s="37"/>
-      <c r="O20" s="37"/>
-      <c r="P20" s="37"/>
+      <c r="N20" s="37">
+        <v>100</v>
+      </c>
+      <c r="O20" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P20" s="37">
+        <v>2.9499999999999998E-2</v>
+      </c>
       <c r="Q20" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.9499999999999997</v>
       </c>
       <c r="R20" s="41"/>
     </row>
@@ -2311,10 +2664,14 @@
       <c r="H21" s="39" t="s">
         <v>134</v>
       </c>
-      <c r="I21" s="39"/>
-      <c r="J21" s="39"/>
+      <c r="I21" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J21" s="39" t="s">
+        <v>186</v>
+      </c>
       <c r="K21" s="40" t="s">
-        <v>85</v>
+        <v>186</v>
       </c>
       <c r="L21" s="39">
         <v>1</v>
@@ -2323,12 +2680,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N21" s="39"/>
-      <c r="O21" s="39"/>
-      <c r="P21" s="39"/>
+      <c r="N21" s="39">
+        <v>25</v>
+      </c>
+      <c r="O21" s="61" t="s">
+        <v>204</v>
+      </c>
+      <c r="P21" s="39">
+        <v>2.09</v>
+      </c>
       <c r="Q21" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>52.25</v>
       </c>
       <c r="R21" s="42"/>
     </row>
@@ -2356,10 +2719,14 @@
       <c r="H22" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="I22" s="37"/>
-      <c r="J22" s="37"/>
+      <c r="I22" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J22" s="37" t="s">
+        <v>205</v>
+      </c>
       <c r="K22" s="38" t="s">
-        <v>110</v>
+        <v>186</v>
       </c>
       <c r="L22" s="37">
         <v>1</v>
@@ -2368,12 +2735,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N22" s="37"/>
-      <c r="O22" s="37"/>
-      <c r="P22" s="37"/>
+      <c r="N22" s="37">
+        <v>25</v>
+      </c>
+      <c r="O22" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P22" s="37">
+        <v>9.8500000000000004E-2</v>
+      </c>
       <c r="Q22" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.4624999999999999</v>
       </c>
       <c r="R22" s="41"/>
     </row>
@@ -2401,10 +2774,14 @@
       <c r="H23" s="39" t="s">
         <v>136</v>
       </c>
-      <c r="I23" s="39"/>
-      <c r="J23" s="39"/>
+      <c r="I23" s="39" t="s">
+        <v>206</v>
+      </c>
+      <c r="J23" s="39" t="s">
+        <v>207</v>
+      </c>
       <c r="K23" s="40" t="s">
-        <v>111</v>
+        <v>186</v>
       </c>
       <c r="L23" s="39">
         <v>1</v>
@@ -2413,12 +2790,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N23" s="39"/>
-      <c r="O23" s="39"/>
-      <c r="P23" s="39"/>
+      <c r="N23" s="39">
+        <v>30</v>
+      </c>
+      <c r="O23" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P23" s="39">
+        <v>4.2200000000000001E-2</v>
+      </c>
       <c r="Q23" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.266</v>
       </c>
       <c r="R23" s="42"/>
     </row>
@@ -2446,10 +2829,14 @@
       <c r="H24" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="I24" s="37"/>
-      <c r="J24" s="37"/>
+      <c r="I24" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J24" s="37" t="s">
+        <v>186</v>
+      </c>
       <c r="K24" s="38" t="s">
-        <v>88</v>
+        <v>186</v>
       </c>
       <c r="L24" s="37">
         <v>1</v>
@@ -2458,12 +2845,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N24" s="37"/>
-      <c r="O24" s="37"/>
-      <c r="P24" s="37"/>
+      <c r="N24" s="37">
+        <v>25</v>
+      </c>
+      <c r="O24" s="60" t="s">
+        <v>208</v>
+      </c>
+      <c r="P24" s="37">
+        <v>0.30840000000000001</v>
+      </c>
       <c r="Q24" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7.71</v>
       </c>
       <c r="R24" s="41"/>
     </row>
@@ -2491,10 +2884,14 @@
       <c r="H25" s="39" t="s">
         <v>138</v>
       </c>
-      <c r="I25" s="39"/>
-      <c r="J25" s="39"/>
+      <c r="I25" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J25" s="39" t="s">
+        <v>209</v>
+      </c>
       <c r="K25" s="40" t="s">
-        <v>112</v>
+        <v>186</v>
       </c>
       <c r="L25" s="39">
         <v>2</v>
@@ -2503,12 +2900,18 @@
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="N25" s="39"/>
-      <c r="O25" s="39"/>
-      <c r="P25" s="39"/>
+      <c r="N25" s="39">
+        <v>60</v>
+      </c>
+      <c r="O25" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P25" s="39">
+        <v>3.4799999999999998E-2</v>
+      </c>
       <c r="Q25" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.0880000000000001</v>
       </c>
       <c r="R25" s="42"/>
     </row>
@@ -2536,8 +2939,12 @@
       <c r="H26" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="I26" s="37"/>
-      <c r="J26" s="37"/>
+      <c r="I26" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J26" s="37" t="s">
+        <v>210</v>
+      </c>
       <c r="K26" s="38" t="s">
         <v>156</v>
       </c>
@@ -2548,12 +2955,18 @@
         <f t="shared" si="2"/>
         <v>800</v>
       </c>
-      <c r="N26" s="37"/>
-      <c r="O26" s="37"/>
-      <c r="P26" s="37"/>
+      <c r="N26" s="37">
+        <v>900</v>
+      </c>
+      <c r="O26" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P26" s="37">
+        <v>8.9999999999999998E-4</v>
+      </c>
       <c r="Q26" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.80999999999999994</v>
       </c>
       <c r="R26" s="41"/>
     </row>
@@ -2581,8 +2994,12 @@
       <c r="H27" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="I27" s="39"/>
-      <c r="J27" s="39"/>
+      <c r="I27" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J27" s="39" t="s">
+        <v>211</v>
+      </c>
       <c r="K27" s="40" t="s">
         <v>157</v>
       </c>
@@ -2593,12 +3010,18 @@
         <f t="shared" si="2"/>
         <v>140</v>
       </c>
-      <c r="N27" s="39"/>
-      <c r="O27" s="39"/>
-      <c r="P27" s="39"/>
+      <c r="N27" s="39">
+        <v>200</v>
+      </c>
+      <c r="O27" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P27" s="39">
+        <v>1.1999999999999999E-3</v>
+      </c>
       <c r="Q27" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="R27" s="42"/>
     </row>
@@ -2626,8 +3049,12 @@
       <c r="H28" s="37" t="s">
         <v>139</v>
       </c>
-      <c r="I28" s="37"/>
-      <c r="J28" s="37"/>
+      <c r="I28" s="37" t="s">
+        <v>212</v>
+      </c>
+      <c r="J28" s="37" t="s">
+        <v>213</v>
+      </c>
       <c r="K28" s="38" t="s">
         <v>158</v>
       </c>
@@ -2638,12 +3065,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N28" s="37"/>
-      <c r="O28" s="37"/>
-      <c r="P28" s="37"/>
+      <c r="N28" s="37">
+        <v>100</v>
+      </c>
+      <c r="O28" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P28" s="37">
+        <v>2.0999999999999999E-3</v>
+      </c>
       <c r="Q28" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="R28" s="41"/>
     </row>
@@ -2671,8 +3104,12 @@
       <c r="H29" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="I29" s="39"/>
-      <c r="J29" s="39"/>
+      <c r="I29" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J29" s="39" t="s">
+        <v>214</v>
+      </c>
       <c r="K29" s="40" t="s">
         <v>159</v>
       </c>
@@ -2683,12 +3120,18 @@
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="N29" s="39"/>
-      <c r="O29" s="39"/>
-      <c r="P29" s="39"/>
+      <c r="N29" s="39">
+        <v>100</v>
+      </c>
+      <c r="O29" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P29" s="39">
+        <v>1.4E-3</v>
+      </c>
       <c r="Q29" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.13999999999999999</v>
       </c>
       <c r="R29" s="42"/>
     </row>
@@ -2716,8 +3159,12 @@
       <c r="H30" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="I30" s="37"/>
-      <c r="J30" s="37"/>
+      <c r="I30" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J30" s="37" t="s">
+        <v>215</v>
+      </c>
       <c r="K30" s="38" t="s">
         <v>160</v>
       </c>
@@ -2728,12 +3175,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N30" s="37"/>
-      <c r="O30" s="37"/>
-      <c r="P30" s="37"/>
+      <c r="N30" s="37">
+        <v>100</v>
+      </c>
+      <c r="O30" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P30" s="37">
+        <v>1.4E-3</v>
+      </c>
       <c r="Q30" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.13999999999999999</v>
       </c>
       <c r="R30" s="41"/>
     </row>
@@ -2761,8 +3214,12 @@
       <c r="H31" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="I31" s="39"/>
-      <c r="J31" s="39"/>
+      <c r="I31" s="39" t="s">
+        <v>216</v>
+      </c>
+      <c r="J31" s="39" t="s">
+        <v>217</v>
+      </c>
       <c r="K31" s="40" t="s">
         <v>161</v>
       </c>
@@ -2773,12 +3230,18 @@
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="N31" s="39"/>
-      <c r="O31" s="39"/>
-      <c r="P31" s="39"/>
+      <c r="N31" s="39">
+        <v>50</v>
+      </c>
+      <c r="O31" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P31" s="39">
+        <v>1.01E-2</v>
+      </c>
       <c r="Q31" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.505</v>
       </c>
       <c r="R31" s="42"/>
     </row>
@@ -2788,40 +3251,56 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="37" t="s">
+      <c r="C32" s="76" t="s">
         <v>92</v>
       </c>
-      <c r="D32" s="37" t="s">
+      <c r="D32" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="E32" s="38" t="s">
+      <c r="E32" s="77" t="s">
         <v>66</v>
       </c>
-      <c r="F32" s="37" t="s">
+      <c r="F32" s="76" t="s">
         <v>92</v>
       </c>
-      <c r="G32" s="38"/>
-      <c r="H32" s="37"/>
-      <c r="I32" s="37"/>
-      <c r="J32" s="37"/>
-      <c r="K32" s="38" t="s">
-        <v>92</v>
-      </c>
-      <c r="L32" s="37">
+      <c r="G32" s="77" t="s">
+        <v>186</v>
+      </c>
+      <c r="H32" s="76" t="s">
+        <v>186</v>
+      </c>
+      <c r="I32" s="76" t="s">
+        <v>186</v>
+      </c>
+      <c r="J32" s="76" t="s">
+        <v>186</v>
+      </c>
+      <c r="K32" s="77" t="s">
+        <v>186</v>
+      </c>
+      <c r="L32" s="76">
         <v>8</v>
       </c>
-      <c r="M32" s="37">
+      <c r="M32" s="76">
         <f t="shared" si="2"/>
         <v>160</v>
       </c>
-      <c r="N32" s="37"/>
-      <c r="O32" s="37"/>
-      <c r="P32" s="37"/>
-      <c r="Q32" s="41">
+      <c r="N32" s="76">
+        <v>160</v>
+      </c>
+      <c r="O32" s="76" t="s">
+        <v>186</v>
+      </c>
+      <c r="P32" s="76">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="78">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="R32" s="41"/>
+      <c r="R32" s="78" t="s">
+        <v>218</v>
+      </c>
     </row>
     <row r="33" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
@@ -2847,10 +3326,14 @@
       <c r="H33" s="39" t="s">
         <v>140</v>
       </c>
-      <c r="I33" s="39"/>
-      <c r="J33" s="39"/>
+      <c r="I33" s="39" t="s">
+        <v>219</v>
+      </c>
+      <c r="J33" s="39" t="s">
+        <v>220</v>
+      </c>
       <c r="K33" s="40" t="s">
-        <v>93</v>
+        <v>186</v>
       </c>
       <c r="L33" s="39">
         <v>1</v>
@@ -2859,149 +3342,191 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N33" s="39"/>
-      <c r="O33" s="39"/>
-      <c r="P33" s="39"/>
+      <c r="N33" s="39">
+        <v>30</v>
+      </c>
+      <c r="O33" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P33" s="39">
+        <v>4.9599999999999998E-2</v>
+      </c>
       <c r="Q33" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.488</v>
       </c>
       <c r="R33" s="42"/>
     </row>
-    <row r="34" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="53">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="37" t="s">
+      <c r="C34" s="65" t="s">
         <v>173</v>
       </c>
-      <c r="D34" s="37" t="s">
+      <c r="D34" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="E34" s="38" t="s">
+      <c r="E34" s="66" t="s">
         <v>68</v>
       </c>
-      <c r="F34" s="37" t="s">
+      <c r="F34" s="65" t="s">
         <v>176</v>
       </c>
-      <c r="G34" s="38" t="s">
+      <c r="G34" s="66" t="s">
         <v>119</v>
       </c>
-      <c r="H34" s="37" t="s">
+      <c r="H34" s="65" t="s">
         <v>141</v>
       </c>
-      <c r="I34" s="37"/>
-      <c r="J34" s="37"/>
-      <c r="K34" s="38" t="s">
-        <v>119</v>
-      </c>
-      <c r="L34" s="37">
+      <c r="I34" s="65" t="s">
+        <v>221</v>
+      </c>
+      <c r="J34" s="65" t="s">
+        <v>222</v>
+      </c>
+      <c r="K34" s="66" t="s">
+        <v>186</v>
+      </c>
+      <c r="L34" s="65">
         <v>1</v>
       </c>
-      <c r="M34" s="37">
+      <c r="M34" s="65">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N34" s="37"/>
-      <c r="O34" s="37"/>
-      <c r="P34" s="37"/>
-      <c r="Q34" s="41">
+      <c r="N34" s="65">
+        <v>22</v>
+      </c>
+      <c r="O34" s="67" t="s">
+        <v>188</v>
+      </c>
+      <c r="P34" s="65">
+        <v>10.947699999999999</v>
+      </c>
+      <c r="Q34" s="68">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R34" s="41"/>
-    </row>
-    <row r="35" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>240.84939999999997</v>
+      </c>
+      <c r="R34" s="73" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="B35" s="53">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="39" t="s">
+      <c r="C35" s="79" t="s">
         <v>173</v>
       </c>
-      <c r="D35" s="39" t="s">
+      <c r="D35" s="79" t="s">
         <v>36</v>
       </c>
-      <c r="E35" s="40" t="s">
+      <c r="E35" s="80" t="s">
         <v>69</v>
       </c>
-      <c r="F35" s="39" t="s">
+      <c r="F35" s="79" t="s">
         <v>94</v>
       </c>
-      <c r="G35" s="40" t="s">
+      <c r="G35" s="80" t="s">
         <v>120</v>
       </c>
-      <c r="H35" s="39" t="s">
+      <c r="H35" s="79" t="s">
         <v>142</v>
       </c>
-      <c r="I35" s="39"/>
-      <c r="J35" s="39"/>
-      <c r="K35" s="40" t="s">
-        <v>120</v>
-      </c>
-      <c r="L35" s="39">
+      <c r="I35" s="79" t="s">
+        <v>224</v>
+      </c>
+      <c r="J35" s="79" t="s">
+        <v>225</v>
+      </c>
+      <c r="K35" s="80" t="s">
+        <v>186</v>
+      </c>
+      <c r="L35" s="79">
         <v>1</v>
       </c>
-      <c r="M35" s="39">
+      <c r="M35" s="79">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N35" s="39"/>
-      <c r="O35" s="39"/>
-      <c r="P35" s="39"/>
-      <c r="Q35" s="42">
+      <c r="N35" s="79">
+        <v>22</v>
+      </c>
+      <c r="O35" s="81" t="s">
+        <v>188</v>
+      </c>
+      <c r="P35" s="79">
+        <v>3.0078999999999998</v>
+      </c>
+      <c r="Q35" s="82">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R35" s="42"/>
-    </row>
-    <row r="36" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>66.1738</v>
+      </c>
+      <c r="R35" s="73" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1"/>
       <c r="B36" s="53">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="37" t="s">
+      <c r="C36" s="65" t="s">
         <v>173</v>
       </c>
-      <c r="D36" s="37" t="s">
+      <c r="D36" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="E36" s="38" t="s">
+      <c r="E36" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="F36" s="37" t="s">
+      <c r="F36" s="65" t="s">
         <v>95</v>
       </c>
-      <c r="G36" s="38" t="s">
+      <c r="G36" s="66" t="s">
         <v>121</v>
       </c>
-      <c r="H36" s="37" t="s">
+      <c r="H36" s="65" t="s">
         <v>143</v>
       </c>
-      <c r="I36" s="37"/>
-      <c r="J36" s="37"/>
-      <c r="K36" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="L36" s="37">
+      <c r="I36" s="65" t="s">
+        <v>226</v>
+      </c>
+      <c r="J36" s="65" t="s">
+        <v>227</v>
+      </c>
+      <c r="K36" s="66" t="s">
+        <v>186</v>
+      </c>
+      <c r="L36" s="65">
         <v>1</v>
       </c>
-      <c r="M36" s="37">
+      <c r="M36" s="65">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N36" s="37"/>
-      <c r="O36" s="37"/>
-      <c r="P36" s="37"/>
-      <c r="Q36" s="41">
+      <c r="N36" s="65">
+        <v>22</v>
+      </c>
+      <c r="O36" s="67" t="s">
+        <v>188</v>
+      </c>
+      <c r="P36" s="65">
+        <v>4.2937000000000003</v>
+      </c>
+      <c r="Q36" s="68">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R36" s="41"/>
+        <v>94.461400000000012</v>
+      </c>
+      <c r="R36" s="73" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="37" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1"/>
@@ -3027,10 +3552,14 @@
       <c r="H37" s="39" t="s">
         <v>144</v>
       </c>
-      <c r="I37" s="39"/>
-      <c r="J37" s="39"/>
+      <c r="I37" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J37" s="39" t="s">
+        <v>186</v>
+      </c>
       <c r="K37" s="40" t="s">
-        <v>122</v>
+        <v>186</v>
       </c>
       <c r="L37" s="39">
         <v>1</v>
@@ -3039,12 +3568,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N37" s="39"/>
-      <c r="O37" s="39"/>
-      <c r="P37" s="39"/>
+      <c r="N37" s="39">
+        <v>22</v>
+      </c>
+      <c r="O37" s="61" t="s">
+        <v>229</v>
+      </c>
+      <c r="P37" s="39">
+        <v>10.6416</v>
+      </c>
       <c r="Q37" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>234.11520000000002</v>
       </c>
       <c r="R37" s="42"/>
     </row>
@@ -3072,10 +3607,14 @@
       <c r="H38" s="37" t="s">
         <v>142</v>
       </c>
-      <c r="I38" s="37"/>
-      <c r="J38" s="37"/>
+      <c r="I38" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J38" s="37" t="s">
+        <v>230</v>
+      </c>
       <c r="K38" s="38" t="s">
-        <v>123</v>
+        <v>186</v>
       </c>
       <c r="L38" s="37">
         <v>1</v>
@@ -3084,12 +3623,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N38" s="37"/>
-      <c r="O38" s="37"/>
-      <c r="P38" s="37"/>
+      <c r="N38" s="37">
+        <v>22</v>
+      </c>
+      <c r="O38" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P38" s="37">
+        <v>0.3337</v>
+      </c>
       <c r="Q38" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7.3414000000000001</v>
       </c>
       <c r="R38" s="41"/>
     </row>
@@ -3117,10 +3662,14 @@
       <c r="H39" s="39" t="s">
         <v>145</v>
       </c>
-      <c r="I39" s="39"/>
-      <c r="J39" s="39"/>
+      <c r="I39" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J39" s="39" t="s">
+        <v>186</v>
+      </c>
       <c r="K39" s="40" t="s">
-        <v>124</v>
+        <v>186</v>
       </c>
       <c r="L39" s="39">
         <v>1</v>
@@ -3129,12 +3678,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N39" s="39"/>
-      <c r="O39" s="39"/>
-      <c r="P39" s="39"/>
+      <c r="N39" s="39">
+        <v>22</v>
+      </c>
+      <c r="O39" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P39" s="39">
+        <v>1.06</v>
+      </c>
       <c r="Q39" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>23.32</v>
       </c>
       <c r="R39" s="42"/>
     </row>
@@ -3162,10 +3717,14 @@
       <c r="H40" s="37" t="s">
         <v>133</v>
       </c>
-      <c r="I40" s="37"/>
-      <c r="J40" s="37"/>
+      <c r="I40" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J40" s="37" t="s">
+        <v>231</v>
+      </c>
       <c r="K40" s="38" t="s">
-        <v>125</v>
+        <v>186</v>
       </c>
       <c r="L40" s="37">
         <v>1</v>
@@ -3174,12 +3733,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N40" s="37"/>
-      <c r="O40" s="37"/>
-      <c r="P40" s="37"/>
+      <c r="N40" s="37">
+        <v>22</v>
+      </c>
+      <c r="O40" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="P40" s="37">
+        <v>0.77</v>
+      </c>
       <c r="Q40" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>16.940000000000001</v>
       </c>
       <c r="R40" s="41"/>
     </row>
@@ -3207,8 +3772,12 @@
       <c r="H41" s="39" t="s">
         <v>146</v>
       </c>
-      <c r="I41" s="39"/>
-      <c r="J41" s="39"/>
+      <c r="I41" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J41" s="39" t="s">
+        <v>186</v>
+      </c>
       <c r="K41" s="40" t="s">
         <v>162</v>
       </c>
@@ -3219,12 +3788,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N41" s="39"/>
-      <c r="O41" s="39"/>
-      <c r="P41" s="39"/>
+      <c r="N41" s="39">
+        <v>22</v>
+      </c>
+      <c r="O41" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="P41" s="39">
+        <v>0.499</v>
+      </c>
       <c r="Q41" s="42">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>10.978</v>
       </c>
       <c r="R41" s="42"/>
     </row>
@@ -3252,10 +3827,14 @@
       <c r="H42" s="37" t="s">
         <v>147</v>
       </c>
-      <c r="I42" s="37"/>
-      <c r="J42" s="58"/>
+      <c r="I42" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="J42" s="58" t="s">
+        <v>186</v>
+      </c>
       <c r="K42" s="38" t="s">
-        <v>101</v>
+        <v>232</v>
       </c>
       <c r="L42" s="37">
         <v>1</v>
@@ -3264,12 +3843,18 @@
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N42" s="37"/>
-      <c r="O42" s="37"/>
-      <c r="P42" s="37"/>
+      <c r="N42" s="37">
+        <v>22</v>
+      </c>
+      <c r="O42" s="60" t="s">
+        <v>204</v>
+      </c>
+      <c r="P42" s="37">
+        <v>0.69</v>
+      </c>
       <c r="Q42" s="41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>15.18</v>
       </c>
       <c r="R42" s="41"/>
     </row>
@@ -3290,9 +3875,14 @@
       <c r="L43" s="36"/>
       <c r="M43" s="36"/>
       <c r="N43" s="36"/>
-      <c r="O43" s="36"/>
-      <c r="P43" s="36"/>
-      <c r="Q43" s="36"/>
+      <c r="O43" s="83" t="s">
+        <v>233</v>
+      </c>
+      <c r="P43" s="84"/>
+      <c r="Q43" s="83">
+        <f>SUM(Q10:Q42)</f>
+        <v>795.37520000000006</v>
+      </c>
       <c r="R43" s="44"/>
     </row>
     <row r="44" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -3312,9 +3902,14 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
-      <c r="O44" s="9"/>
-      <c r="P44" s="9"/>
-      <c r="Q44" s="9"/>
+      <c r="O44" s="85" t="s">
+        <v>234</v>
+      </c>
+      <c r="P44" s="86"/>
+      <c r="Q44" s="85">
+        <f>Q43/20</f>
+        <v>39.76876</v>
+      </c>
       <c r="R44" s="45"/>
     </row>
   </sheetData>
@@ -3325,9 +3920,39 @@
   <hyperlinks>
     <hyperlink ref="O10" r:id="rId1"/>
     <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O12" r:id="rId3"/>
+    <hyperlink ref="O13" r:id="rId4"/>
+    <hyperlink ref="O14" r:id="rId5"/>
+    <hyperlink ref="O15" r:id="rId6"/>
+    <hyperlink ref="O16" r:id="rId7"/>
+    <hyperlink ref="O17" r:id="rId8"/>
+    <hyperlink ref="O18" r:id="rId9"/>
+    <hyperlink ref="O19" r:id="rId10"/>
+    <hyperlink ref="O20" r:id="rId11"/>
+    <hyperlink ref="O21" r:id="rId12"/>
+    <hyperlink ref="O22" r:id="rId13"/>
+    <hyperlink ref="O23" r:id="rId14"/>
+    <hyperlink ref="O24" r:id="rId15"/>
+    <hyperlink ref="O25" r:id="rId16"/>
+    <hyperlink ref="O26" r:id="rId17"/>
+    <hyperlink ref="O27" r:id="rId18"/>
+    <hyperlink ref="O28" r:id="rId19"/>
+    <hyperlink ref="O29" r:id="rId20"/>
+    <hyperlink ref="O30" r:id="rId21"/>
+    <hyperlink ref="O31" r:id="rId22"/>
+    <hyperlink ref="O33" r:id="rId23"/>
+    <hyperlink ref="O34" r:id="rId24"/>
+    <hyperlink ref="O35" r:id="rId25"/>
+    <hyperlink ref="O36" r:id="rId26"/>
+    <hyperlink ref="O37" r:id="rId27"/>
+    <hyperlink ref="O38" r:id="rId28"/>
+    <hyperlink ref="O39" r:id="rId29"/>
+    <hyperlink ref="O40" r:id="rId30"/>
+    <hyperlink ref="O41" r:id="rId31"/>
+    <hyperlink ref="O42" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
-  <drawing r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId33"/>
+  <drawing r:id="rId34"/>
 </worksheet>
 </file>
</xml_diff>